<commit_message>
Replace all customer data with Vaniday beauty/wellness scenario
</commit_message>
<xml_diff>
--- a/dummy_invoice_upload.xlsx
+++ b/dummy_invoice_upload.xlsx
@@ -441,13 +441,13 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B2" t="str">
-        <v>Acme Learning Centre</v>
+        <v>Luxe Hair Studio</v>
       </c>
       <c r="C2" t="str">
-        <v>accounts@acmelearning.sg</v>
+        <v>bookings@luxehairstudio.sg</v>
       </c>
       <c r="D2" t="str">
         <v>2026-05-01</v>
@@ -456,13 +456,13 @@
         <v>2026-05-15</v>
       </c>
       <c r="F2" t="str">
-        <v>Math enrichment session</v>
+        <v>Balayage hair coloring</v>
       </c>
       <c r="G2">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>45.5</v>
+        <v>185</v>
       </c>
       <c r="I2" t="str">
         <v>Sent</v>
@@ -470,13 +470,13 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B3" t="str">
-        <v>Acme Learning Centre</v>
+        <v>Luxe Hair Studio</v>
       </c>
       <c r="C3" t="str">
-        <v>accounts@acmelearning.sg</v>
+        <v>bookings@luxehairstudio.sg</v>
       </c>
       <c r="D3" t="str">
         <v>2026-05-01</v>
@@ -485,13 +485,13 @@
         <v>2026-05-15</v>
       </c>
       <c r="F3" t="str">
-        <v>Learning materials</v>
+        <v>Olaplex hair treatment</v>
       </c>
       <c r="G3">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>8.9</v>
+        <v>65</v>
       </c>
       <c r="I3" t="str">
         <v>Sent</v>
@@ -499,13 +499,13 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B4" t="str">
-        <v>BrightPath Tuition</v>
+        <v>The Nail Artistry</v>
       </c>
       <c r="C4" t="str">
-        <v>finance@brightpath.sg</v>
+        <v>hello@thenailartistry.sg</v>
       </c>
       <c r="D4" t="str">
         <v>2026-05-03</v>
@@ -514,13 +514,13 @@
         <v>2026-05-17</v>
       </c>
       <c r="F4" t="str">
-        <v>Science workshop</v>
+        <v>Gel manicure session</v>
       </c>
       <c r="G4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H4">
-        <v>38.75</v>
+        <v>48</v>
       </c>
       <c r="I4" t="str">
         <v>Viewed</v>
@@ -528,13 +528,13 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B5" t="str">
-        <v>BrightPath Tuition</v>
+        <v>The Nail Artistry</v>
       </c>
       <c r="C5" t="str">
-        <v>finance@brightpath.sg</v>
+        <v>hello@thenailartistry.sg</v>
       </c>
       <c r="D5" t="str">
         <v>2026-05-03</v>
@@ -543,13 +543,13 @@
         <v>2026-05-17</v>
       </c>
       <c r="F5" t="str">
-        <v>Assessment pack</v>
+        <v>Nail art add-on</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H5">
-        <v>6.5</v>
+        <v>25</v>
       </c>
       <c r="I5" t="str">
         <v>Viewed</v>
@@ -557,13 +557,13 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B6" t="str">
-        <v>Nova Skills Academy</v>
+        <v>Serenity Spa &amp; Wellness</v>
       </c>
       <c r="C6" t="str">
-        <v>billing@novaskills.sg</v>
+        <v>reservations@serenityspa.sg</v>
       </c>
       <c r="D6" t="str">
         <v>2026-05-05</v>
@@ -572,13 +572,13 @@
         <v>2026-05-19</v>
       </c>
       <c r="F6" t="str">
-        <v>Excel automation training</v>
+        <v>Full body massage (90 min)</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>52</v>
+        <v>158</v>
       </c>
       <c r="I6" t="str">
         <v>Paid</v>
@@ -586,13 +586,13 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B7" t="str">
-        <v>Nova Skills Academy</v>
+        <v>Serenity Spa &amp; Wellness</v>
       </c>
       <c r="C7" t="str">
-        <v>billing@novaskills.sg</v>
+        <v>reservations@serenityspa.sg</v>
       </c>
       <c r="D7" t="str">
         <v>2026-05-05</v>
@@ -601,13 +601,13 @@
         <v>2026-05-19</v>
       </c>
       <c r="F7" t="str">
-        <v>Trainer travel allowance</v>
+        <v>Aromatherapy upgrade</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I7" t="str">
         <v>Paid</v>
@@ -615,13 +615,13 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B8" t="str">
-        <v>Summit Corporate Training</v>
+        <v>Glow Aesthetics Clinic</v>
       </c>
       <c r="C8" t="str">
-        <v>payables@summittraining.sg</v>
+        <v>appointments@glowaesthetics.sg</v>
       </c>
       <c r="D8" t="str">
         <v>2026-04-20</v>
@@ -630,13 +630,13 @@
         <v>2026-05-04</v>
       </c>
       <c r="F8" t="str">
-        <v>Leadership bootcamp</v>
+        <v>Hydrafacial treatment</v>
       </c>
       <c r="G8">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>64</v>
+        <v>280</v>
       </c>
       <c r="I8" t="str">
         <v>Overdue</v>
@@ -644,13 +644,13 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B9" t="str">
-        <v>Summit Corporate Training</v>
+        <v>Glow Aesthetics Clinic</v>
       </c>
       <c r="C9" t="str">
-        <v>payables@summittraining.sg</v>
+        <v>appointments@glowaesthetics.sg</v>
       </c>
       <c r="D9" t="str">
         <v>2026-04-20</v>
@@ -659,13 +659,13 @@
         <v>2026-05-04</v>
       </c>
       <c r="F9" t="str">
-        <v>Course handbook</v>
+        <v>LED light therapy add-on</v>
       </c>
       <c r="G9">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>7.25</v>
+        <v>85</v>
       </c>
       <c r="I9" t="str">
         <v>Overdue</v>
@@ -673,13 +673,13 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B10" t="str">
-        <v>Urban Tech Institute</v>
+        <v>Brow &amp; Lash Bar</v>
       </c>
       <c r="C10" t="str">
-        <v>admin@urbantech.edu.sg</v>
+        <v>info@browlashbar.sg</v>
       </c>
       <c r="D10" t="str">
         <v>2026-05-08</v>
@@ -688,13 +688,13 @@
         <v>2026-05-22</v>
       </c>
       <c r="F10" t="str">
-        <v>Coding lab support</v>
+        <v>Eyebrow embroidery</v>
       </c>
       <c r="G10">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H10">
-        <v>72.5</v>
+        <v>388</v>
       </c>
       <c r="I10" t="str">
         <v>Draft</v>
@@ -702,13 +702,13 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B11" t="str">
-        <v>Urban Tech Institute</v>
+        <v>Brow &amp; Lash Bar</v>
       </c>
       <c r="C11" t="str">
-        <v>admin@urbantech.edu.sg</v>
+        <v>info@browlashbar.sg</v>
       </c>
       <c r="D11" t="str">
         <v>2026-05-08</v>
@@ -717,13 +717,13 @@
         <v>2026-05-22</v>
       </c>
       <c r="F11" t="str">
-        <v>USB learning kit</v>
+        <v>Lash lift &amp; tint</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11">
-        <v>12.4</v>
+        <v>78</v>
       </c>
       <c r="I11" t="str">
         <v>Draft</v>
@@ -731,13 +731,13 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B12" t="str">
-        <v>Acme Learning Centre</v>
+        <v>Luxe Hair Studio</v>
       </c>
       <c r="C12" t="str">
-        <v>accounts@acmelearning.sg</v>
+        <v>bookings@luxehairstudio.sg</v>
       </c>
       <c r="D12" t="str">
         <v>2026-05-10</v>
@@ -746,13 +746,13 @@
         <v>2026-05-24</v>
       </c>
       <c r="F12" t="str">
-        <v>Holiday programme</v>
+        <v>Keratin smoothing treatment</v>
       </c>
       <c r="G12">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H12">
-        <v>49.9</v>
+        <v>220</v>
       </c>
       <c r="I12" t="str">
         <v>Paid</v>
@@ -760,13 +760,13 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B13" t="str">
-        <v>BrightPath Tuition</v>
+        <v>The Nail Artistry</v>
       </c>
       <c r="C13" t="str">
-        <v>finance@brightpath.sg</v>
+        <v>hello@thenailartistry.sg</v>
       </c>
       <c r="D13" t="str">
         <v>2026-05-12</v>
@@ -775,13 +775,13 @@
         <v>2026-05-26</v>
       </c>
       <c r="F13" t="str">
-        <v>English clinic</v>
+        <v>Classic pedicure</v>
       </c>
       <c r="G13">
         <v>9</v>
       </c>
       <c r="H13">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="I13" t="str">
         <v>Sent</v>
@@ -789,13 +789,13 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B14" t="str">
-        <v>BrightPath Tuition</v>
+        <v>The Nail Artistry</v>
       </c>
       <c r="C14" t="str">
-        <v>finance@brightpath.sg</v>
+        <v>hello@thenailartistry.sg</v>
       </c>
       <c r="D14" t="str">
         <v>2026-05-12</v>
@@ -804,13 +804,13 @@
         <v>2026-05-26</v>
       </c>
       <c r="F14" t="str">
-        <v>Worksheet bundle</v>
+        <v>Paraffin wax treatment</v>
       </c>
       <c r="G14">
         <v>9</v>
       </c>
       <c r="H14">
-        <v>5.75</v>
+        <v>22</v>
       </c>
       <c r="I14" t="str">
         <v>Sent</v>
@@ -818,13 +818,13 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B15" t="str">
-        <v>Nova Skills Academy</v>
+        <v>Serenity Spa &amp; Wellness</v>
       </c>
       <c r="C15" t="str">
-        <v>billing@novaskills.sg</v>
+        <v>reservations@serenityspa.sg</v>
       </c>
       <c r="D15" t="str">
         <v>2026-05-14</v>
@@ -833,13 +833,13 @@
         <v>2026-05-28</v>
       </c>
       <c r="F15" t="str">
-        <v>Power BI fundamentals</v>
+        <v>Hot stone massage</v>
       </c>
       <c r="G15">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>58</v>
+        <v>188</v>
       </c>
       <c r="I15" t="str">
         <v>Sent</v>
@@ -847,13 +847,13 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B16" t="str">
-        <v>Nova Skills Academy</v>
+        <v>Serenity Spa &amp; Wellness</v>
       </c>
       <c r="C16" t="str">
-        <v>billing@novaskills.sg</v>
+        <v>reservations@serenityspa.sg</v>
       </c>
       <c r="D16" t="str">
         <v>2026-05-14</v>
@@ -862,13 +862,13 @@
         <v>2026-05-28</v>
       </c>
       <c r="F16" t="str">
-        <v>Certificate printing</v>
+        <v>Complimentary herbal tea set</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H16">
-        <v>3.5</v>
+        <v>12</v>
       </c>
       <c r="I16" t="str">
         <v>Sent</v>

</xml_diff>